<commit_message>
Updated list of files for Photo Gallery
updated Photos.html and images list spreadsheet of files to load
</commit_message>
<xml_diff>
--- a/assets/js/RentOasis-images.xlsx
+++ b/assets/js/RentOasis-images.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Isx529wiGq4+NMhwF00HK+mNidaTRHjKC51a9WVDS7c="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="wOEi/NJ0iqRB9eoLAQFNa9iWgG2OMkI5vlbwUOPkkeQ="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="92">
   <si>
     <t>Filename</t>
   </si>
@@ -256,13 +256,49 @@
   </si>
   <si>
     <t>livingroom6.JPG</t>
+  </si>
+  <si>
+    <t>Fancy-Living_Room.webp</t>
+  </si>
+  <si>
+    <t>Fancy-Bedroom.webp</t>
+  </si>
+  <si>
+    <t>Fancy-Bedroom2.webp</t>
+  </si>
+  <si>
+    <t>Fancy-Living_Room2.webp</t>
+  </si>
+  <si>
+    <t>Fancy-Bathroom.webp</t>
+  </si>
+  <si>
+    <t>Bathroom Hallway</t>
+  </si>
+  <si>
+    <t>Fancy-Dollhouse_View.webp</t>
+  </si>
+  <si>
+    <t>3D Model</t>
+  </si>
+  <si>
+    <t>Interior, Floor Plan</t>
+  </si>
+  <si>
+    <t>Fancy-Bedroom3.webp</t>
+  </si>
+  <si>
+    <t>Fancy-Bedroom4.webp</t>
+  </si>
+  <si>
+    <t>Fancy-Kitchen1.webp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -291,6 +327,11 @@
       <u/>
       <color rgb="FF0000FF"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -306,7 +347,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -320,6 +361,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
@@ -537,7 +584,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="19.38"/>
+    <col customWidth="1" min="1" max="1" width="22.38"/>
     <col customWidth="1" min="2" max="2" width="27.25"/>
     <col customWidth="1" min="3" max="3" width="22.0"/>
     <col customWidth="1" min="4" max="5" width="26.5"/>
@@ -592,13 +639,13 @@
         <v>7</v>
       </c>
       <c r="B2" s="4" t="str">
-        <f t="shared" ref="B2:B39" si="1">"https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/" &amp; A2 &amp; "?v=" &amp; RANDBETWEEN(1,999999)
+        <f t="shared" ref="B2:B48" si="1">"https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/" &amp; A2 &amp; "?v=" &amp; RANDBETWEEN(1,999999)
 </f>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/sofa-rent123.jpg?v=121424</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/sofa-rent123.jpg?v=64817</v>
       </c>
       <c r="C2" s="3" t="str">
-        <f t="shared" ref="C2:C39" si="2">IMAGE(B2,1)</f>
-        <v>Loading...</v>
+        <f t="shared" ref="C2:C48" si="2">IMAGE(B2,1)</f>
+        <v/>
       </c>
       <c r="D2" s="5" t="s">
         <v>8</v>
@@ -619,11 +666,11 @@
       </c>
       <c r="B3" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroom1.jpg?v=267307</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroom1.jpg?v=179540</v>
       </c>
       <c r="C3" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D3" s="5" t="s">
         <v>11</v>
@@ -644,11 +691,11 @@
       </c>
       <c r="B4" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroom2.jpg?v=231626</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroom2.jpg?v=632488</v>
       </c>
       <c r="C4" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D4" s="5" t="s">
         <v>11</v>
@@ -669,11 +716,11 @@
       </c>
       <c r="B5" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/hallway1.jpg?v=835105</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/hallway1.jpg?v=105095</v>
       </c>
       <c r="C5" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D5" s="5" t="s">
         <v>15</v>
@@ -694,11 +741,11 @@
       </c>
       <c r="B6" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/hallway2.jpg?v=153779</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/hallway2.jpg?v=985714</v>
       </c>
       <c r="C6" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D6" s="5" t="s">
         <v>15</v>
@@ -719,11 +766,11 @@
       </c>
       <c r="B7" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroomfront.jpg?v=351066</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroomfront.jpg?v=53680</v>
       </c>
       <c r="C7" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D7" s="5" t="s">
         <v>11</v>
@@ -744,11 +791,11 @@
       </c>
       <c r="B8" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroomdoor.jpg?v=919532</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroomdoor.jpg?v=372231</v>
       </c>
       <c r="C8" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D8" s="5" t="s">
         <v>11</v>
@@ -769,11 +816,11 @@
       </c>
       <c r="B9" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroomfront2.jpg?v=823482</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroomfront2.jpg?v=60507</v>
       </c>
       <c r="C9" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D9" s="5" t="s">
         <v>11</v>
@@ -794,11 +841,11 @@
       </c>
       <c r="B10" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom1.jpg?v=314136</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom1.jpg?v=444649</v>
       </c>
       <c r="C10" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D10" s="5" t="s">
         <v>22</v>
@@ -819,11 +866,11 @@
       </c>
       <c r="B11" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom2.jpg?v=956637</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom2.jpg?v=339630</v>
       </c>
       <c r="C11" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D11" s="5" t="s">
         <v>22</v>
@@ -844,11 +891,11 @@
       </c>
       <c r="B12" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom3.jpg?v=520443</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom3.jpg?v=235268</v>
       </c>
       <c r="C12" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D12" s="5" t="s">
         <v>22</v>
@@ -869,11 +916,11 @@
       </c>
       <c r="B13" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom4.jpg?v=83281</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom4.jpg?v=420285</v>
       </c>
       <c r="C13" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D13" s="5" t="s">
         <v>22</v>
@@ -894,11 +941,11 @@
       </c>
       <c r="B14" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchen1.jpg?v=881091</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchen1.jpg?v=178618</v>
       </c>
       <c r="C14" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D14" s="5" t="s">
         <v>27</v>
@@ -919,11 +966,11 @@
       </c>
       <c r="B15" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchen2.jpg?v=973924</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchen2.jpg?v=211118</v>
       </c>
       <c r="C15" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D15" s="5" t="s">
         <v>27</v>
@@ -944,11 +991,11 @@
       </c>
       <c r="B16" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchen3.jpg?v=79410</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchen3.jpg?v=439500</v>
       </c>
       <c r="C16" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D16" s="5" t="s">
         <v>27</v>
@@ -969,11 +1016,11 @@
       </c>
       <c r="B17" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bathroom.jpg?v=79510</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bathroom.jpg?v=428558</v>
       </c>
       <c r="C17" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D17" s="5" t="s">
         <v>32</v>
@@ -994,11 +1041,11 @@
       </c>
       <c r="B18" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/sofa.jpg?v=491301</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/sofa.jpg?v=642531</v>
       </c>
       <c r="C18" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D18" s="5" t="s">
         <v>22</v>
@@ -1019,11 +1066,11 @@
       </c>
       <c r="B19" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/301anacostia.png?v=326508</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/301anacostia.png?v=749538</v>
       </c>
       <c r="C19" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D19" s="5" t="s">
         <v>36</v>
@@ -1044,11 +1091,11 @@
       </c>
       <c r="B20" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/305.jpeg?v=492257</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/305.jpeg?v=477298</v>
       </c>
       <c r="C20" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D20" s="5" t="s">
         <v>39</v>
@@ -1069,11 +1116,11 @@
       </c>
       <c r="B21" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/3517.png?v=867504</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/3517.png?v=688894</v>
       </c>
       <c r="C21" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D21" s="5" t="s">
         <v>42</v>
@@ -1094,11 +1141,11 @@
       </c>
       <c r="B22" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/303.png?v=324141</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/303.png?v=505763</v>
       </c>
       <c r="C22" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D22" s="5" t="s">
         <v>45</v>
@@ -1119,11 +1166,11 @@
       </c>
       <c r="B23" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/307.png?v=536587</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/307.png?v=187824</v>
       </c>
       <c r="C23" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D23" s="5" t="s">
         <v>48</v>
@@ -1144,11 +1191,11 @@
       </c>
       <c r="B24" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/3515.png?v=21223</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/3515.png?v=463197</v>
       </c>
       <c r="C24" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D24" s="5" t="s">
         <v>51</v>
@@ -1169,11 +1216,11 @@
       </c>
       <c r="B25" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/3519.png?v=711477</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/3519.png?v=689975</v>
       </c>
       <c r="C25" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D25" s="5" t="s">
         <v>54</v>
@@ -1194,11 +1241,11 @@
       </c>
       <c r="B26" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/3521.png?v=478697</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/3521.png?v=11536</v>
       </c>
       <c r="C26" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D26" s="5" t="s">
         <v>57</v>
@@ -1219,11 +1266,11 @@
       </c>
       <c r="B27" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom-furniture1.png?v=840171</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom-furniture1.png?v=611938</v>
       </c>
       <c r="C27" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D27" s="5" t="s">
         <v>60</v>
@@ -1244,11 +1291,11 @@
       </c>
       <c r="B28" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroom1furniture.png?v=211743</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/bedroom1furniture.png?v=68490</v>
       </c>
       <c r="C28" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D28" s="5" t="s">
         <v>60</v>
@@ -1269,11 +1316,11 @@
       </c>
       <c r="B29" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchensink1.JPG?v=749359</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchensink1.JPG?v=449621</v>
       </c>
       <c r="C29" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D29" s="5" t="s">
         <v>64</v>
@@ -1294,11 +1341,11 @@
       </c>
       <c r="B30" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/hallwayclosets1.JPG?v=719748</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/hallwayclosets1.JPG?v=744218</v>
       </c>
       <c r="C30" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D30" s="5" t="s">
         <v>15</v>
@@ -1319,11 +1366,11 @@
       </c>
       <c r="B31" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchenstove1.JPG?v=668092</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchenstove1.JPG?v=743459</v>
       </c>
       <c r="C31" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D31" s="5" t="s">
         <v>67</v>
@@ -1344,11 +1391,11 @@
       </c>
       <c r="B32" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/hallwayclosets3.JPG?v=737138</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/hallwayclosets3.JPG?v=519941</v>
       </c>
       <c r="C32" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D32" s="5" t="s">
         <v>15</v>
@@ -1369,11 +1416,11 @@
       </c>
       <c r="B33" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchennook1.JPG?v=529777</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchennook1.JPG?v=24149</v>
       </c>
       <c r="C33" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D33" s="5" t="s">
         <v>70</v>
@@ -1394,11 +1441,11 @@
       </c>
       <c r="B34" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchenstove2.JPG?v=446166</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchenstove2.JPG?v=502925</v>
       </c>
       <c r="C34" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D34" s="5" t="s">
         <v>67</v>
@@ -1419,11 +1466,11 @@
       </c>
       <c r="B35" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchensink2.JPG?v=868003</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchensink2.JPG?v=25301</v>
       </c>
       <c r="C35" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D35" s="5" t="s">
         <v>64</v>
@@ -1444,11 +1491,11 @@
       </c>
       <c r="B36" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchencorner1.JPG?v=952863</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/kitchencorner1.JPG?v=496271</v>
       </c>
       <c r="C36" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D36" s="5" t="s">
         <v>74</v>
@@ -1469,11 +1516,11 @@
       </c>
       <c r="B37" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/diningroom1.JPG?v=509678</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/diningroom1.JPG?v=556794</v>
       </c>
       <c r="C37" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D37" s="5" t="s">
         <v>76</v>
@@ -1494,11 +1541,11 @@
       </c>
       <c r="B38" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom5.JPG?v=818163</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom5.JPG?v=789392</v>
       </c>
       <c r="C38" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D38" s="5" t="s">
         <v>22</v>
@@ -1519,11 +1566,11 @@
       </c>
       <c r="B39" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom6.JPG?v=258325</v>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/livingroom6.JPG?v=737545</v>
       </c>
       <c r="C39" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Loading...</v>
+        <v/>
       </c>
       <c r="D39" s="5" t="s">
         <v>22</v>
@@ -1538,1272 +1585,1188 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="B40" s="6"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="B41" s="6"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="6"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="B43" s="6"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
-      <c r="B44" s="6"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="B45" s="6"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="B46" s="6"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
-      <c r="B47" s="6"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5"/>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
-      <c r="B48" s="6"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
+    <row r="40" ht="142.5" customHeight="1">
+      <c r="A40" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B40" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Living_Room.webp?v=268730</v>
+      </c>
+      <c r="C40" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G40" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" ht="142.5" customHeight="1">
+      <c r="A41" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B41" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Bedroom.webp?v=871949</v>
+      </c>
+      <c r="C41" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" ht="142.5" customHeight="1">
+      <c r="A42" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Bedroom2.webp?v=883900</v>
+      </c>
+      <c r="C42" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" ht="142.5" customHeight="1">
+      <c r="A43" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B43" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Living_Room2.webp?v=281488</v>
+      </c>
+      <c r="C43" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G43" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" ht="142.5" customHeight="1">
+      <c r="A44" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B44" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Bathroom.webp?v=101087</v>
+      </c>
+      <c r="C44" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G44" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" ht="142.5" customHeight="1">
+      <c r="A45" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B45" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Dollhouse_View.webp?v=361212</v>
+      </c>
+      <c r="C45" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G45" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" ht="142.5" customHeight="1">
+      <c r="A46" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B46" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Bedroom3.webp?v=605115</v>
+      </c>
+      <c r="C46" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" ht="142.5" customHeight="1">
+      <c r="A47" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B47" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Bedroom4.webp?v=87352</v>
+      </c>
+      <c r="C47" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" ht="142.5" customHeight="1">
+      <c r="A48" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B48" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>https://raw.githubusercontent.com/RightGuy/rentoasis-site/main/assets/images/Fancy-Kitchen1.webp?v=749485</v>
+      </c>
+      <c r="C48" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G48" s="5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="B49" s="6"/>
+      <c r="B49" s="8"/>
       <c r="D49" s="5"/>
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="B50" s="6"/>
+      <c r="B50" s="8"/>
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="B51" s="6"/>
+      <c r="B51" s="8"/>
       <c r="D51" s="5"/>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="B52" s="6"/>
+      <c r="B52" s="8"/>
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="B53" s="6"/>
+      <c r="B53" s="8"/>
       <c r="D53" s="5"/>
       <c r="E53" s="5"/>
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="B54" s="6"/>
+      <c r="B54" s="8"/>
       <c r="D54" s="5"/>
       <c r="E54" s="5"/>
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="B55" s="6"/>
+      <c r="B55" s="8"/>
       <c r="D55" s="5"/>
       <c r="E55" s="5"/>
       <c r="F55" s="5"/>
       <c r="G55" s="5"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="B56" s="6"/>
+      <c r="B56" s="8"/>
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
       <c r="F56" s="5"/>
       <c r="G56" s="5"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="B57" s="6"/>
+      <c r="B57" s="8"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
       <c r="F57" s="5"/>
       <c r="G57" s="5"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="B58" s="6"/>
+      <c r="B58" s="8"/>
       <c r="D58" s="5"/>
       <c r="E58" s="5"/>
       <c r="F58" s="5"/>
       <c r="G58" s="5"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="B59" s="6"/>
+      <c r="B59" s="8"/>
       <c r="D59" s="5"/>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="B60" s="6"/>
+      <c r="B60" s="8"/>
       <c r="D60" s="5"/>
       <c r="E60" s="5"/>
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="B61" s="6"/>
+      <c r="B61" s="8"/>
       <c r="D61" s="5"/>
       <c r="E61" s="5"/>
       <c r="F61" s="5"/>
       <c r="G61" s="5"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="B62" s="6"/>
+      <c r="B62" s="8"/>
       <c r="D62" s="5"/>
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
       <c r="G62" s="5"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="B63" s="6"/>
+      <c r="B63" s="8"/>
       <c r="D63" s="5"/>
       <c r="E63" s="5"/>
       <c r="F63" s="5"/>
       <c r="G63" s="5"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="B64" s="6"/>
+      <c r="B64" s="8"/>
       <c r="D64" s="5"/>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="B65" s="6"/>
+      <c r="B65" s="8"/>
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
       <c r="G65" s="5"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="B66" s="6"/>
+      <c r="B66" s="8"/>
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
       <c r="G66" s="5"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="B67" s="6"/>
+      <c r="B67" s="8"/>
       <c r="D67" s="5"/>
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
       <c r="G67" s="5"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="B68" s="6"/>
+      <c r="B68" s="8"/>
       <c r="D68" s="5"/>
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
       <c r="G68" s="5"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="B69" s="6"/>
+      <c r="B69" s="8"/>
       <c r="D69" s="5"/>
       <c r="E69" s="5"/>
       <c r="F69" s="5"/>
       <c r="G69" s="5"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="B70" s="6"/>
+      <c r="B70" s="8"/>
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
       <c r="G70" s="5"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="B71" s="6"/>
+      <c r="B71" s="8"/>
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
       <c r="F71" s="5"/>
       <c r="G71" s="5"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="B72" s="6"/>
+      <c r="B72" s="8"/>
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
       <c r="F72" s="5"/>
       <c r="G72" s="5"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="B73" s="6"/>
+      <c r="B73" s="8"/>
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
       <c r="F73" s="5"/>
       <c r="G73" s="5"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="B74" s="6"/>
+      <c r="B74" s="8"/>
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
       <c r="F74" s="5"/>
       <c r="G74" s="5"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="B75" s="6"/>
+      <c r="B75" s="8"/>
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
       <c r="F75" s="5"/>
       <c r="G75" s="5"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="B76" s="6"/>
+      <c r="B76" s="8"/>
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
       <c r="G76" s="5"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="B77" s="6"/>
+      <c r="B77" s="8"/>
       <c r="D77" s="5"/>
       <c r="E77" s="5"/>
       <c r="F77" s="5"/>
       <c r="G77" s="5"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="B78" s="6"/>
+      <c r="B78" s="8"/>
       <c r="D78" s="5"/>
       <c r="E78" s="5"/>
       <c r="F78" s="5"/>
       <c r="G78" s="5"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="B79" s="6"/>
+      <c r="B79" s="8"/>
       <c r="D79" s="5"/>
       <c r="E79" s="5"/>
       <c r="F79" s="5"/>
       <c r="G79" s="5"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="B80" s="6"/>
+      <c r="B80" s="8"/>
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="5"/>
       <c r="G80" s="5"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="B81" s="6"/>
+      <c r="B81" s="8"/>
       <c r="D81" s="5"/>
       <c r="E81" s="5"/>
       <c r="F81" s="5"/>
       <c r="G81" s="5"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="B82" s="6"/>
+      <c r="B82" s="8"/>
       <c r="D82" s="5"/>
       <c r="E82" s="5"/>
       <c r="F82" s="5"/>
       <c r="G82" s="5"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="B83" s="6"/>
+      <c r="B83" s="8"/>
       <c r="D83" s="5"/>
       <c r="E83" s="5"/>
       <c r="F83" s="5"/>
       <c r="G83" s="5"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="B84" s="6"/>
+      <c r="B84" s="8"/>
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
       <c r="F84" s="5"/>
       <c r="G84" s="5"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="B85" s="6"/>
+      <c r="B85" s="8"/>
       <c r="D85" s="5"/>
       <c r="E85" s="5"/>
       <c r="F85" s="5"/>
       <c r="G85" s="5"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="B86" s="6"/>
+      <c r="B86" s="8"/>
       <c r="D86" s="5"/>
       <c r="E86" s="5"/>
       <c r="F86" s="5"/>
       <c r="G86" s="5"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="B87" s="6"/>
+      <c r="B87" s="8"/>
       <c r="D87" s="5"/>
       <c r="E87" s="5"/>
       <c r="F87" s="5"/>
       <c r="G87" s="5"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
-      <c r="B88" s="6"/>
+      <c r="B88" s="8"/>
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
       <c r="F88" s="5"/>
       <c r="G88" s="5"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="B89" s="6"/>
+      <c r="B89" s="8"/>
       <c r="D89" s="5"/>
       <c r="E89" s="5"/>
       <c r="F89" s="5"/>
       <c r="G89" s="5"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="B90" s="6"/>
+      <c r="B90" s="8"/>
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
       <c r="F90" s="5"/>
       <c r="G90" s="5"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="B91" s="6"/>
+      <c r="B91" s="8"/>
       <c r="D91" s="5"/>
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
       <c r="G91" s="5"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
-      <c r="B92" s="6"/>
+      <c r="B92" s="8"/>
       <c r="D92" s="5"/>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
       <c r="G92" s="5"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="B93" s="6"/>
+      <c r="B93" s="8"/>
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
       <c r="F93" s="5"/>
       <c r="G93" s="5"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
-      <c r="B94" s="6"/>
+      <c r="B94" s="8"/>
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
       <c r="F94" s="5"/>
       <c r="G94" s="5"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
-      <c r="B95" s="6"/>
+      <c r="B95" s="8"/>
       <c r="D95" s="5"/>
       <c r="E95" s="5"/>
       <c r="F95" s="5"/>
       <c r="G95" s="5"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
-      <c r="B96" s="6"/>
+      <c r="B96" s="8"/>
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
       <c r="F96" s="5"/>
       <c r="G96" s="5"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="B97" s="6"/>
+      <c r="B97" s="8"/>
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
       <c r="G97" s="5"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
-      <c r="B98" s="6"/>
+      <c r="B98" s="8"/>
       <c r="D98" s="5"/>
       <c r="E98" s="5"/>
       <c r="F98" s="5"/>
       <c r="G98" s="5"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
-      <c r="B99" s="6"/>
+      <c r="B99" s="8"/>
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
       <c r="F99" s="5"/>
       <c r="G99" s="5"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
-      <c r="B100" s="6"/>
+      <c r="B100" s="8"/>
       <c r="D100" s="5"/>
       <c r="E100" s="5"/>
       <c r="F100" s="5"/>
       <c r="G100" s="5"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
-      <c r="B101" s="6"/>
+      <c r="B101" s="8"/>
       <c r="D101" s="5"/>
       <c r="E101" s="5"/>
       <c r="F101" s="5"/>
       <c r="G101" s="5"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
-      <c r="B102" s="6"/>
+      <c r="B102" s="8"/>
       <c r="D102" s="5"/>
       <c r="E102" s="5"/>
       <c r="F102" s="5"/>
       <c r="G102" s="5"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
-      <c r="B103" s="6"/>
+      <c r="B103" s="8"/>
       <c r="D103" s="5"/>
       <c r="E103" s="5"/>
       <c r="F103" s="5"/>
       <c r="G103" s="5"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
-      <c r="B104" s="6"/>
+      <c r="B104" s="8"/>
       <c r="D104" s="5"/>
       <c r="E104" s="5"/>
       <c r="F104" s="5"/>
       <c r="G104" s="5"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
-      <c r="B105" s="6"/>
+      <c r="B105" s="8"/>
       <c r="D105" s="5"/>
       <c r="E105" s="5"/>
       <c r="F105" s="5"/>
       <c r="G105" s="5"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="B106" s="6"/>
+      <c r="B106" s="8"/>
       <c r="D106" s="5"/>
       <c r="E106" s="5"/>
       <c r="F106" s="5"/>
       <c r="G106" s="5"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="B107" s="6"/>
+      <c r="B107" s="8"/>
       <c r="D107" s="5"/>
       <c r="E107" s="5"/>
       <c r="F107" s="5"/>
       <c r="G107" s="5"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
-      <c r="B108" s="6"/>
+      <c r="B108" s="8"/>
       <c r="D108" s="5"/>
       <c r="E108" s="5"/>
       <c r="F108" s="5"/>
       <c r="G108" s="5"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
-      <c r="B109" s="6"/>
+      <c r="B109" s="8"/>
       <c r="D109" s="5"/>
       <c r="E109" s="5"/>
       <c r="F109" s="5"/>
       <c r="G109" s="5"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
-      <c r="B110" s="6"/>
+      <c r="B110" s="8"/>
       <c r="D110" s="5"/>
       <c r="E110" s="5"/>
       <c r="F110" s="5"/>
       <c r="G110" s="5"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
-      <c r="B111" s="6"/>
+      <c r="B111" s="8"/>
       <c r="D111" s="5"/>
       <c r="E111" s="5"/>
       <c r="F111" s="5"/>
       <c r="G111" s="5"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
-      <c r="B112" s="6"/>
+      <c r="B112" s="8"/>
       <c r="D112" s="5"/>
       <c r="E112" s="5"/>
       <c r="F112" s="5"/>
       <c r="G112" s="5"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
-      <c r="B113" s="6"/>
+      <c r="B113" s="8"/>
       <c r="D113" s="5"/>
       <c r="E113" s="5"/>
       <c r="F113" s="5"/>
       <c r="G113" s="5"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
-      <c r="B114" s="6"/>
+      <c r="B114" s="8"/>
       <c r="D114" s="5"/>
       <c r="E114" s="5"/>
       <c r="F114" s="5"/>
       <c r="G114" s="5"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
-      <c r="B115" s="6"/>
+      <c r="B115" s="8"/>
       <c r="D115" s="5"/>
       <c r="E115" s="5"/>
       <c r="F115" s="5"/>
       <c r="G115" s="5"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="B116" s="6"/>
+      <c r="B116" s="8"/>
       <c r="D116" s="5"/>
       <c r="E116" s="5"/>
       <c r="F116" s="5"/>
       <c r="G116" s="5"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
-      <c r="B117" s="6"/>
+      <c r="B117" s="8"/>
       <c r="D117" s="5"/>
       <c r="E117" s="5"/>
       <c r="F117" s="5"/>
       <c r="G117" s="5"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
-      <c r="B118" s="6"/>
+      <c r="B118" s="8"/>
       <c r="D118" s="5"/>
       <c r="E118" s="5"/>
       <c r="F118" s="5"/>
       <c r="G118" s="5"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
-      <c r="B119" s="6"/>
+      <c r="B119" s="8"/>
       <c r="D119" s="5"/>
       <c r="E119" s="5"/>
       <c r="F119" s="5"/>
       <c r="G119" s="5"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
-      <c r="B120" s="6"/>
+      <c r="B120" s="8"/>
       <c r="D120" s="5"/>
       <c r="E120" s="5"/>
       <c r="F120" s="5"/>
       <c r="G120" s="5"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
-      <c r="B121" s="6"/>
+      <c r="B121" s="8"/>
       <c r="D121" s="5"/>
       <c r="E121" s="5"/>
       <c r="F121" s="5"/>
       <c r="G121" s="5"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
-      <c r="B122" s="6"/>
+      <c r="B122" s="8"/>
       <c r="D122" s="5"/>
       <c r="E122" s="5"/>
       <c r="F122" s="5"/>
       <c r="G122" s="5"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
-      <c r="B123" s="6"/>
+      <c r="B123" s="8"/>
       <c r="D123" s="5"/>
       <c r="E123" s="5"/>
       <c r="F123" s="5"/>
       <c r="G123" s="5"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
-      <c r="B124" s="6"/>
+      <c r="B124" s="8"/>
       <c r="D124" s="5"/>
       <c r="E124" s="5"/>
       <c r="F124" s="5"/>
       <c r="G124" s="5"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
-      <c r="B125" s="6"/>
+      <c r="B125" s="8"/>
       <c r="D125" s="5"/>
       <c r="E125" s="5"/>
       <c r="F125" s="5"/>
       <c r="G125" s="5"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
-      <c r="B126" s="6"/>
+      <c r="B126" s="8"/>
       <c r="D126" s="5"/>
       <c r="E126" s="5"/>
       <c r="F126" s="5"/>
       <c r="G126" s="5"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
-      <c r="B127" s="6"/>
+      <c r="B127" s="8"/>
       <c r="D127" s="5"/>
       <c r="E127" s="5"/>
       <c r="F127" s="5"/>
       <c r="G127" s="5"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
-      <c r="B128" s="6"/>
+      <c r="B128" s="8"/>
       <c r="D128" s="5"/>
       <c r="E128" s="5"/>
       <c r="F128" s="5"/>
       <c r="G128" s="5"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
-      <c r="B129" s="6"/>
+      <c r="B129" s="8"/>
       <c r="D129" s="5"/>
       <c r="E129" s="5"/>
       <c r="F129" s="5"/>
       <c r="G129" s="5"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
-      <c r="B130" s="6"/>
+      <c r="B130" s="8"/>
       <c r="D130" s="5"/>
       <c r="E130" s="5"/>
       <c r="F130" s="5"/>
       <c r="G130" s="5"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
-      <c r="B131" s="6"/>
+      <c r="B131" s="8"/>
       <c r="D131" s="5"/>
       <c r="E131" s="5"/>
       <c r="F131" s="5"/>
       <c r="G131" s="5"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
-      <c r="B132" s="6"/>
+      <c r="B132" s="8"/>
       <c r="D132" s="5"/>
       <c r="E132" s="5"/>
       <c r="F132" s="5"/>
       <c r="G132" s="5"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
-      <c r="B133" s="6"/>
+      <c r="B133" s="8"/>
       <c r="D133" s="5"/>
       <c r="E133" s="5"/>
       <c r="F133" s="5"/>
       <c r="G133" s="5"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
-      <c r="B134" s="6"/>
+      <c r="B134" s="8"/>
       <c r="D134" s="5"/>
       <c r="E134" s="5"/>
       <c r="F134" s="5"/>
       <c r="G134" s="5"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
-      <c r="B135" s="6"/>
+      <c r="B135" s="8"/>
       <c r="D135" s="5"/>
       <c r="E135" s="5"/>
       <c r="F135" s="5"/>
       <c r="G135" s="5"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
-      <c r="B136" s="6"/>
+      <c r="B136" s="8"/>
       <c r="D136" s="5"/>
       <c r="E136" s="5"/>
       <c r="F136" s="5"/>
       <c r="G136" s="5"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
-      <c r="B137" s="6"/>
+      <c r="B137" s="8"/>
       <c r="D137" s="5"/>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
       <c r="G137" s="5"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
-      <c r="B138" s="6"/>
+      <c r="B138" s="8"/>
       <c r="D138" s="5"/>
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
       <c r="G138" s="5"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
-      <c r="B139" s="6"/>
+      <c r="B139" s="8"/>
       <c r="D139" s="5"/>
       <c r="E139" s="5"/>
       <c r="F139" s="5"/>
       <c r="G139" s="5"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
-      <c r="B140" s="6"/>
+      <c r="B140" s="8"/>
       <c r="D140" s="5"/>
       <c r="E140" s="5"/>
       <c r="F140" s="5"/>
       <c r="G140" s="5"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
-      <c r="B141" s="6"/>
+      <c r="B141" s="8"/>
       <c r="D141" s="5"/>
       <c r="E141" s="5"/>
       <c r="F141" s="5"/>
       <c r="G141" s="5"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
-      <c r="B142" s="6"/>
+      <c r="B142" s="8"/>
       <c r="D142" s="5"/>
       <c r="E142" s="5"/>
       <c r="F142" s="5"/>
       <c r="G142" s="5"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
-      <c r="B143" s="6"/>
+      <c r="B143" s="8"/>
       <c r="D143" s="5"/>
       <c r="E143" s="5"/>
       <c r="F143" s="5"/>
       <c r="G143" s="5"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
-      <c r="B144" s="6"/>
+      <c r="B144" s="8"/>
       <c r="D144" s="5"/>
       <c r="E144" s="5"/>
       <c r="F144" s="5"/>
       <c r="G144" s="5"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
-      <c r="B145" s="6"/>
+      <c r="B145" s="8"/>
       <c r="D145" s="5"/>
       <c r="E145" s="5"/>
       <c r="F145" s="5"/>
       <c r="G145" s="5"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
-      <c r="B146" s="6"/>
+      <c r="B146" s="8"/>
       <c r="D146" s="5"/>
       <c r="E146" s="5"/>
       <c r="F146" s="5"/>
       <c r="G146" s="5"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
-      <c r="B147" s="6"/>
+      <c r="B147" s="8"/>
       <c r="D147" s="5"/>
       <c r="E147" s="5"/>
       <c r="F147" s="5"/>
       <c r="G147" s="5"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
-      <c r="B148" s="6"/>
+      <c r="B148" s="8"/>
       <c r="D148" s="5"/>
       <c r="E148" s="5"/>
       <c r="F148" s="5"/>
       <c r="G148" s="5"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
-      <c r="B149" s="6"/>
+      <c r="B149" s="8"/>
       <c r="D149" s="5"/>
       <c r="E149" s="5"/>
       <c r="F149" s="5"/>
       <c r="G149" s="5"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
-      <c r="B150" s="6"/>
+      <c r="B150" s="8"/>
       <c r="D150" s="5"/>
       <c r="E150" s="5"/>
       <c r="F150" s="5"/>
       <c r="G150" s="5"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
-      <c r="B151" s="6"/>
+      <c r="B151" s="8"/>
       <c r="D151" s="5"/>
       <c r="E151" s="5"/>
       <c r="F151" s="5"/>
       <c r="G151" s="5"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
-      <c r="B152" s="6"/>
+      <c r="B152" s="8"/>
       <c r="D152" s="5"/>
       <c r="E152" s="5"/>
       <c r="F152" s="5"/>
       <c r="G152" s="5"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
-      <c r="B153" s="6"/>
+      <c r="B153" s="8"/>
       <c r="D153" s="5"/>
       <c r="E153" s="5"/>
       <c r="F153" s="5"/>
       <c r="G153" s="5"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
-      <c r="B154" s="6"/>
+      <c r="B154" s="8"/>
       <c r="D154" s="5"/>
       <c r="E154" s="5"/>
       <c r="F154" s="5"/>
       <c r="G154" s="5"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
-      <c r="B155" s="6"/>
+      <c r="B155" s="8"/>
       <c r="D155" s="5"/>
       <c r="E155" s="5"/>
       <c r="F155" s="5"/>
       <c r="G155" s="5"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
-      <c r="B156" s="6"/>
+      <c r="B156" s="8"/>
       <c r="D156" s="5"/>
       <c r="E156" s="5"/>
       <c r="F156" s="5"/>
       <c r="G156" s="5"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
-      <c r="B157" s="6"/>
+      <c r="B157" s="8"/>
       <c r="D157" s="5"/>
       <c r="E157" s="5"/>
       <c r="F157" s="5"/>
       <c r="G157" s="5"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
-      <c r="B158" s="6"/>
+      <c r="B158" s="8"/>
       <c r="D158" s="5"/>
       <c r="E158" s="5"/>
       <c r="F158" s="5"/>
       <c r="G158" s="5"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
-      <c r="B159" s="6"/>
+      <c r="B159" s="8"/>
       <c r="D159" s="5"/>
       <c r="E159" s="5"/>
       <c r="F159" s="5"/>
       <c r="G159" s="5"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
-      <c r="B160" s="6"/>
+      <c r="B160" s="8"/>
       <c r="D160" s="5"/>
       <c r="E160" s="5"/>
       <c r="F160" s="5"/>
       <c r="G160" s="5"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
-      <c r="B161" s="6"/>
+      <c r="B161" s="8"/>
       <c r="D161" s="5"/>
       <c r="E161" s="5"/>
       <c r="F161" s="5"/>
       <c r="G161" s="5"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
-      <c r="B162" s="6"/>
+      <c r="B162" s="8"/>
       <c r="D162" s="5"/>
       <c r="E162" s="5"/>
       <c r="F162" s="5"/>
       <c r="G162" s="5"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
-      <c r="B163" s="6"/>
+      <c r="B163" s="8"/>
       <c r="D163" s="5"/>
       <c r="E163" s="5"/>
       <c r="F163" s="5"/>
       <c r="G163" s="5"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
-      <c r="B164" s="6"/>
+      <c r="B164" s="8"/>
       <c r="D164" s="5"/>
       <c r="E164" s="5"/>
       <c r="F164" s="5"/>
       <c r="G164" s="5"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
-      <c r="B165" s="6"/>
+      <c r="B165" s="8"/>
       <c r="D165" s="5"/>
       <c r="E165" s="5"/>
       <c r="F165" s="5"/>
       <c r="G165" s="5"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
-      <c r="B166" s="6"/>
+      <c r="B166" s="8"/>
       <c r="D166" s="5"/>
       <c r="E166" s="5"/>
       <c r="F166" s="5"/>
       <c r="G166" s="5"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
-      <c r="B167" s="6"/>
+      <c r="B167" s="8"/>
       <c r="D167" s="5"/>
       <c r="E167" s="5"/>
       <c r="F167" s="5"/>
       <c r="G167" s="5"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
-      <c r="B168" s="6"/>
+      <c r="B168" s="8"/>
       <c r="D168" s="5"/>
       <c r="E168" s="5"/>
       <c r="F168" s="5"/>
       <c r="G168" s="5"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
-      <c r="B169" s="6"/>
+      <c r="B169" s="8"/>
       <c r="D169" s="5"/>
       <c r="E169" s="5"/>
       <c r="F169" s="5"/>
       <c r="G169" s="5"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
-      <c r="B170" s="6"/>
+      <c r="B170" s="8"/>
       <c r="D170" s="5"/>
       <c r="E170" s="5"/>
       <c r="F170" s="5"/>
       <c r="G170" s="5"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
-      <c r="B171" s="6"/>
+      <c r="B171" s="8"/>
       <c r="D171" s="5"/>
       <c r="E171" s="5"/>
       <c r="F171" s="5"/>
       <c r="G171" s="5"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
-      <c r="B172" s="6"/>
+      <c r="B172" s="8"/>
       <c r="D172" s="5"/>
       <c r="E172" s="5"/>
       <c r="F172" s="5"/>
       <c r="G172" s="5"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
-      <c r="B173" s="6"/>
+      <c r="B173" s="8"/>
       <c r="D173" s="5"/>
       <c r="E173" s="5"/>
       <c r="F173" s="5"/>
       <c r="G173" s="5"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
-      <c r="B174" s="6"/>
+      <c r="B174" s="8"/>
       <c r="D174" s="5"/>
       <c r="E174" s="5"/>
       <c r="F174" s="5"/>
       <c r="G174" s="5"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
-      <c r="B175" s="6"/>
+      <c r="B175" s="8"/>
       <c r="D175" s="5"/>
       <c r="E175" s="5"/>
       <c r="F175" s="5"/>
       <c r="G175" s="5"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
-      <c r="B176" s="6"/>
+      <c r="B176" s="8"/>
       <c r="D176" s="5"/>
       <c r="E176" s="5"/>
       <c r="F176" s="5"/>
       <c r="G176" s="5"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
-      <c r="B177" s="6"/>
+      <c r="B177" s="8"/>
       <c r="D177" s="5"/>
       <c r="E177" s="5"/>
       <c r="F177" s="5"/>
       <c r="G177" s="5"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
-      <c r="B178" s="6"/>
+      <c r="B178" s="8"/>
       <c r="D178" s="5"/>
       <c r="E178" s="5"/>
       <c r="F178" s="5"/>
       <c r="G178" s="5"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
-      <c r="B179" s="6"/>
       <c r="D179" s="5"/>
       <c r="E179" s="5"/>
       <c r="F179" s="5"/>
       <c r="G179" s="5"/>
     </row>
-    <row r="180" ht="15.75" customHeight="1">
-      <c r="B180" s="6"/>
-      <c r="D180" s="5"/>
-      <c r="E180" s="5"/>
-      <c r="F180" s="5"/>
-      <c r="G180" s="5"/>
-    </row>
-    <row r="181" ht="15.75" customHeight="1">
-      <c r="B181" s="6"/>
-      <c r="D181" s="5"/>
-      <c r="E181" s="5"/>
-      <c r="F181" s="5"/>
-      <c r="G181" s="5"/>
-    </row>
-    <row r="182" ht="15.75" customHeight="1">
-      <c r="B182" s="6"/>
-      <c r="D182" s="5"/>
-      <c r="E182" s="5"/>
-      <c r="F182" s="5"/>
-      <c r="G182" s="5"/>
-    </row>
-    <row r="183" ht="15.75" customHeight="1">
-      <c r="B183" s="6"/>
-      <c r="D183" s="5"/>
-      <c r="E183" s="5"/>
-      <c r="F183" s="5"/>
-      <c r="G183" s="5"/>
-    </row>
-    <row r="184" ht="15.75" customHeight="1">
-      <c r="B184" s="6"/>
-      <c r="D184" s="5"/>
-      <c r="E184" s="5"/>
-      <c r="F184" s="5"/>
-      <c r="G184" s="5"/>
-    </row>
-    <row r="185" ht="15.75" customHeight="1">
-      <c r="B185" s="6"/>
-      <c r="D185" s="5"/>
-      <c r="E185" s="5"/>
-      <c r="F185" s="5"/>
-      <c r="G185" s="5"/>
-    </row>
-    <row r="186" ht="15.75" customHeight="1">
-      <c r="B186" s="6"/>
-      <c r="D186" s="5"/>
-      <c r="E186" s="5"/>
-      <c r="F186" s="5"/>
-      <c r="G186" s="5"/>
-    </row>
-    <row r="187" ht="15.75" customHeight="1">
-      <c r="B187" s="6"/>
-      <c r="D187" s="5"/>
-      <c r="E187" s="5"/>
-      <c r="F187" s="5"/>
-      <c r="G187" s="5"/>
-    </row>
-    <row r="188" ht="15.75" customHeight="1">
-      <c r="B188" s="6"/>
-      <c r="D188" s="5"/>
-      <c r="E188" s="5"/>
-      <c r="F188" s="5"/>
-      <c r="G188" s="5"/>
-    </row>
-    <row r="189" ht="15.75" customHeight="1">
-      <c r="B189" s="6"/>
-      <c r="D189" s="5"/>
-      <c r="E189" s="5"/>
-      <c r="F189" s="5"/>
-      <c r="G189" s="5"/>
-    </row>
-    <row r="190" ht="15.75" customHeight="1">
-      <c r="B190" s="6"/>
-      <c r="D190" s="5"/>
-      <c r="E190" s="5"/>
-      <c r="F190" s="5"/>
-      <c r="G190" s="5"/>
-    </row>
-    <row r="191" ht="15.75" customHeight="1">
-      <c r="B191" s="6"/>
-      <c r="D191" s="5"/>
-      <c r="E191" s="5"/>
-      <c r="F191" s="5"/>
-      <c r="G191" s="5"/>
-    </row>
-    <row r="192" ht="15.75" customHeight="1">
-      <c r="B192" s="6"/>
-      <c r="D192" s="5"/>
-      <c r="E192" s="5"/>
-      <c r="F192" s="5"/>
-      <c r="G192" s="5"/>
-    </row>
-    <row r="193" ht="15.75" customHeight="1">
-      <c r="B193" s="6"/>
-      <c r="D193" s="5"/>
-      <c r="E193" s="5"/>
-      <c r="F193" s="5"/>
-      <c r="G193" s="5"/>
-    </row>
-    <row r="194" ht="15.75" customHeight="1">
-      <c r="B194" s="6"/>
-      <c r="D194" s="5"/>
-      <c r="E194" s="5"/>
-      <c r="F194" s="5"/>
-      <c r="G194" s="5"/>
-    </row>
-    <row r="195" ht="15.75" customHeight="1">
-      <c r="B195" s="6"/>
-      <c r="D195" s="5"/>
-      <c r="E195" s="5"/>
-      <c r="F195" s="5"/>
-      <c r="G195" s="5"/>
-    </row>
-    <row r="196" ht="15.75" customHeight="1">
-      <c r="B196" s="6"/>
-      <c r="D196" s="5"/>
-      <c r="E196" s="5"/>
-      <c r="F196" s="5"/>
-      <c r="G196" s="5"/>
-    </row>
-    <row r="197" ht="15.75" customHeight="1">
-      <c r="B197" s="6"/>
-      <c r="D197" s="5"/>
-      <c r="E197" s="5"/>
-      <c r="F197" s="5"/>
-      <c r="G197" s="5"/>
-    </row>
-    <row r="198" ht="15.75" customHeight="1">
-      <c r="B198" s="6"/>
-      <c r="D198" s="5"/>
-      <c r="E198" s="5"/>
-      <c r="F198" s="5"/>
-      <c r="G198" s="5"/>
-    </row>
-    <row r="199" ht="15.75" customHeight="1">
-      <c r="B199" s="6"/>
-      <c r="D199" s="5"/>
-      <c r="E199" s="5"/>
-      <c r="F199" s="5"/>
-      <c r="G199" s="5"/>
-    </row>
-    <row r="200" ht="15.75" customHeight="1">
-      <c r="B200" s="6"/>
-      <c r="D200" s="5"/>
-      <c r="E200" s="5"/>
-      <c r="F200" s="5"/>
-      <c r="G200" s="5"/>
-    </row>
-    <row r="201" ht="15.75" customHeight="1">
-      <c r="B201" s="6"/>
-      <c r="D201" s="5"/>
-      <c r="E201" s="5"/>
-      <c r="F201" s="5"/>
-      <c r="G201" s="5"/>
-    </row>
-    <row r="202" ht="15.75" customHeight="1">
-      <c r="B202" s="6"/>
-      <c r="D202" s="5"/>
-      <c r="E202" s="5"/>
-      <c r="F202" s="5"/>
-      <c r="G202" s="5"/>
-    </row>
-    <row r="203" ht="15.75" customHeight="1">
-      <c r="B203" s="6"/>
-      <c r="D203" s="5"/>
-      <c r="E203" s="5"/>
-      <c r="F203" s="5"/>
-      <c r="G203" s="5"/>
-    </row>
-    <row r="204" ht="15.75" customHeight="1">
-      <c r="B204" s="6"/>
-      <c r="D204" s="5"/>
-      <c r="E204" s="5"/>
-      <c r="F204" s="5"/>
-      <c r="G204" s="5"/>
-    </row>
-    <row r="205" ht="15.75" customHeight="1">
-      <c r="B205" s="6"/>
-      <c r="D205" s="5"/>
-      <c r="E205" s="5"/>
-      <c r="F205" s="5"/>
-      <c r="G205" s="5"/>
-    </row>
-    <row r="206" ht="15.75" customHeight="1">
-      <c r="B206" s="6"/>
-      <c r="D206" s="5"/>
-      <c r="E206" s="5"/>
-      <c r="F206" s="5"/>
-      <c r="G206" s="5"/>
-    </row>
-    <row r="207" ht="15.75" customHeight="1">
-      <c r="B207" s="6"/>
-      <c r="D207" s="5"/>
-      <c r="E207" s="5"/>
-      <c r="F207" s="5"/>
-      <c r="G207" s="5"/>
-    </row>
-    <row r="208" ht="15.75" customHeight="1">
-      <c r="B208" s="6"/>
-      <c r="D208" s="5"/>
-      <c r="E208" s="5"/>
-      <c r="F208" s="5"/>
-      <c r="G208" s="5"/>
-    </row>
-    <row r="209" ht="15.75" customHeight="1">
-      <c r="B209" s="6"/>
-      <c r="D209" s="5"/>
-      <c r="E209" s="5"/>
-      <c r="F209" s="5"/>
-      <c r="G209" s="5"/>
-    </row>
-    <row r="210" ht="15.75" customHeight="1">
-      <c r="B210" s="6"/>
-      <c r="D210" s="5"/>
-      <c r="E210" s="5"/>
-      <c r="F210" s="5"/>
-      <c r="G210" s="5"/>
-    </row>
-    <row r="211" ht="15.75" customHeight="1">
-      <c r="B211" s="6"/>
-      <c r="D211" s="5"/>
-      <c r="E211" s="5"/>
-      <c r="F211" s="5"/>
-      <c r="G211" s="5"/>
-    </row>
-    <row r="212" ht="15.75" customHeight="1">
-      <c r="B212" s="6"/>
-      <c r="D212" s="5"/>
-      <c r="E212" s="5"/>
-      <c r="F212" s="5"/>
-      <c r="G212" s="5"/>
-    </row>
-    <row r="213" ht="15.75" customHeight="1">
-      <c r="B213" s="6"/>
-      <c r="D213" s="5"/>
-      <c r="E213" s="5"/>
-      <c r="F213" s="5"/>
-      <c r="G213" s="5"/>
-    </row>
-    <row r="214" ht="15.75" customHeight="1">
-      <c r="B214" s="6"/>
-      <c r="D214" s="5"/>
-      <c r="E214" s="5"/>
-      <c r="F214" s="5"/>
-      <c r="G214" s="5"/>
-    </row>
-    <row r="215" ht="15.75" customHeight="1">
-      <c r="B215" s="6"/>
-      <c r="D215" s="5"/>
-      <c r="E215" s="5"/>
-      <c r="F215" s="5"/>
-      <c r="G215" s="5"/>
-    </row>
-    <row r="216" ht="15.75" customHeight="1">
-      <c r="B216" s="6"/>
-      <c r="D216" s="5"/>
-      <c r="E216" s="5"/>
-      <c r="F216" s="5"/>
-      <c r="G216" s="5"/>
-    </row>
-    <row r="217" ht="15.75" customHeight="1">
-      <c r="B217" s="6"/>
-      <c r="D217" s="5"/>
-      <c r="E217" s="5"/>
-      <c r="F217" s="5"/>
-      <c r="G217" s="5"/>
-    </row>
-    <row r="218" ht="15.75" customHeight="1">
-      <c r="B218" s="6"/>
-      <c r="D218" s="5"/>
-      <c r="E218" s="5"/>
-      <c r="F218" s="5"/>
-      <c r="G218" s="5"/>
-    </row>
-    <row r="219" ht="15.75" customHeight="1">
-      <c r="B219" s="6"/>
-      <c r="D219" s="5"/>
-      <c r="E219" s="5"/>
-      <c r="F219" s="5"/>
-      <c r="G219" s="5"/>
-    </row>
-    <row r="220" ht="15.75" customHeight="1">
-      <c r="D220" s="5"/>
-      <c r="E220" s="5"/>
-      <c r="F220" s="5"/>
-      <c r="G220" s="5"/>
-    </row>
+    <row r="180" ht="15.75" customHeight="1"/>
+    <row r="181" ht="15.75" customHeight="1"/>
+    <row r="182" ht="15.75" customHeight="1"/>
+    <row r="183" ht="15.75" customHeight="1"/>
+    <row r="184" ht="15.75" customHeight="1"/>
+    <row r="185" ht="15.75" customHeight="1"/>
+    <row r="186" ht="15.75" customHeight="1"/>
+    <row r="187" ht="15.75" customHeight="1"/>
+    <row r="188" ht="15.75" customHeight="1"/>
+    <row r="189" ht="15.75" customHeight="1"/>
+    <row r="190" ht="15.75" customHeight="1"/>
+    <row r="191" ht="15.75" customHeight="1"/>
+    <row r="192" ht="15.75" customHeight="1"/>
+    <row r="193" ht="15.75" customHeight="1"/>
+    <row r="194" ht="15.75" customHeight="1"/>
+    <row r="195" ht="15.75" customHeight="1"/>
+    <row r="196" ht="15.75" customHeight="1"/>
+    <row r="197" ht="15.75" customHeight="1"/>
+    <row r="198" ht="15.75" customHeight="1"/>
+    <row r="199" ht="15.75" customHeight="1"/>
+    <row r="200" ht="15.75" customHeight="1"/>
+    <row r="201" ht="15.75" customHeight="1"/>
+    <row r="202" ht="15.75" customHeight="1"/>
+    <row r="203" ht="15.75" customHeight="1"/>
+    <row r="204" ht="15.75" customHeight="1"/>
+    <row r="205" ht="15.75" customHeight="1"/>
+    <row r="206" ht="15.75" customHeight="1"/>
+    <row r="207" ht="15.75" customHeight="1"/>
+    <row r="208" ht="15.75" customHeight="1"/>
+    <row r="209" ht="15.75" customHeight="1"/>
+    <row r="210" ht="15.75" customHeight="1"/>
+    <row r="211" ht="15.75" customHeight="1"/>
+    <row r="212" ht="15.75" customHeight="1"/>
+    <row r="213" ht="15.75" customHeight="1"/>
+    <row r="214" ht="15.75" customHeight="1"/>
+    <row r="215" ht="15.75" customHeight="1"/>
+    <row r="216" ht="15.75" customHeight="1"/>
+    <row r="217" ht="15.75" customHeight="1"/>
+    <row r="218" ht="15.75" customHeight="1"/>
+    <row r="219" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1"/>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1"/>
     <row r="223" ht="15.75" customHeight="1"/>
@@ -3542,47 +3505,6 @@
     <row r="956" ht="15.75" customHeight="1"/>
     <row r="957" ht="15.75" customHeight="1"/>
     <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>